<commit_message>
Complete Amazon automation framework with POM, TestNG, Extent Reports, GitHub Actions, and email reporting
</commit_message>
<xml_diff>
--- a/src/main/resources/testdata/input.xlsx
+++ b/src/main/resources/testdata/input.xlsx
@@ -17,16 +17,16 @@
     <t>SearchKeyword</t>
   </si>
   <si>
-    <t>Toys</t>
+    <t>toys</t>
   </si>
   <si>
-    <t>Books</t>
+    <t>toys under 500</t>
   </si>
   <si>
-    <t>Electronics</t>
+    <t>toys above 500</t>
   </si>
   <si>
-    <t>Mobiles</t>
+    <t>toys for kids</t>
   </si>
 </sst>
 </file>
@@ -79,9 +79,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true"/>
   </cellXfs>
 </styleSheet>
 </file>
@@ -100,22 +104,22 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s" s="0">
+      <c r="A2" t="s" s="2">
         <v>1</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="s" s="0">
+      <c r="A3" t="s" s="3">
         <v>2</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="s" s="0">
+      <c r="A4" t="s" s="4">
         <v>3</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="s" s="0">
+      <c r="A5" t="s" s="5">
         <v>4</v>
       </c>
     </row>

</xml_diff>